<commit_message>
Updating the scripts and corresponding data
</commit_message>
<xml_diff>
--- a/Data/RenamingSequences.xlsx
+++ b/Data/RenamingSequences.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/147a029199edd8ae/PG Materials/Semester3/Structural_Phylogeny/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="196" documentId="8_{F1ECBFBC-D87D-8847-87DE-B5DA96C0745E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{759398F6-9C2F-CE4A-8C1D-0E2D8C1D80C1}"/>
+  <xr:revisionPtr revIDLastSave="198" documentId="8_{F1ECBFBC-D87D-8847-87DE-B5DA96C0745E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F55C15C0-8018-3D4D-8932-565F9D2A7181}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{3D1955E4-042E-8A46-B97E-98CB368699EC}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29280" windowHeight="18880" xr2:uid="{3D1955E4-042E-8A46-B97E-98CB368699EC}"/>
   </bookViews>
   <sheets>
     <sheet name="protein" sheetId="4" r:id="rId1"/>
@@ -3962,10 +3962,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>